<commit_message>
landscape (lucc+bioge16) import data files
</commit_message>
<xml_diff>
--- a/lucas/import_data/dataset_meta/excel/campaign.xlsx
+++ b/lucas/import_data/dataset_meta/excel/campaign.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="48">
   <si>
     <t xml:space="preserve">dataset_id__dataset_name</t>
   </si>
@@ -146,6 +146,24 @@
   </si>
   <si>
     <t xml:space="preserve">foss xds rca,lucas-wetlab-2015</t>
+  </si>
+  <si>
+    <t xml:space="preserve">biogeo16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EU BIOGEO 2016</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.eea.europa.eu/en/datahub/datahubitem-view/11db8d14-f167-4cd5-9205-95638dfd9618</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The biogeographical regions dataset contains the official delineations used in the Habitats Directive (92/43/EEC) and for the EMERALD Network set up under the Convention on the Conservation of European Wildlife and Natural Habitats (Bern Convention).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">map</t>
+  </si>
+  <si>
+    <t xml:space="preserve">compilation</t>
   </si>
 </sst>
 </file>
@@ -155,7 +173,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -180,6 +198,13 @@
     <font>
       <sz val="10"/>
       <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF2F4052"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
@@ -227,7 +252,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -248,6 +273,14 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -257,6 +290,66 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FF00FF00"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008000"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FF808000"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FFC0C0C0"/>
+      <rgbColor rgb="FF808080"/>
+      <rgbColor rgb="FF9999FF"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FF660066"/>
+      <rgbColor rgb="FFFF8080"/>
+      <rgbColor rgb="FF0066CC"/>
+      <rgbColor rgb="FFCCCCFF"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FF00CCFF"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFFFFF99"/>
+      <rgbColor rgb="FF99CCFF"/>
+      <rgbColor rgb="FFFF99CC"/>
+      <rgbColor rgb="FFCC99FF"/>
+      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FF3366FF"/>
+      <rgbColor rgb="FF33CCCC"/>
+      <rgbColor rgb="FF99CC00"/>
+      <rgbColor rgb="FFFFCC00"/>
+      <rgbColor rgb="FFFF9900"/>
+      <rgbColor rgb="FFFF6600"/>
+      <rgbColor rgb="FF666699"/>
+      <rgbColor rgb="FF969696"/>
+      <rgbColor rgb="FF003366"/>
+      <rgbColor rgb="FF339966"/>
+      <rgbColor rgb="FF003300"/>
+      <rgbColor rgb="FF333300"/>
+      <rgbColor rgb="FF993300"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FF333399"/>
+      <rgbColor rgb="FF2F4052"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -268,37 +361,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18a303"/>
+        <a:srgbClr val="18A303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369a3"/>
+        <a:srgbClr val="0369A3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a33e03"/>
+        <a:srgbClr val="A33E03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8e03a3"/>
+        <a:srgbClr val="8E03A3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="c99c00"/>
+        <a:srgbClr val="C99C00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="c9211e"/>
+        <a:srgbClr val="C9211E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ee"/>
+        <a:srgbClr val="0000EE"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551a8b"/>
+        <a:srgbClr val="551A8B"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -371,8 +464,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Z3"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:Z4"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="33.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="27.64"/>
@@ -575,6 +668,59 @@
         <v>41</v>
       </c>
     </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F4" s="1" t="n">
+        <v>20160331</v>
+      </c>
+      <c r="G4" s="1" t="n">
+        <v>20261231</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="J4" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="S4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="T4" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="U4" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="V4" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="W4" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="X4" s="1" t="n">
+        <v>1000</v>
+      </c>
+      <c r="Y4" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="Z4" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="H3" r:id="rId1" display="https://esdac.jrc.ec.europa.eu/content/lucas2015-topsoil-data"/>

</xml_diff>

<commit_message>
Add tag columns and tag-based auto naming
- Add tag columns to dataset, campaign, sampling_log, provision and
  observation_log; add datetime_tag to campaign
- Auto_name concats resolve <table>_id__<table>_<column> by locating the
  record from its name, tag or alias and returning the requested column;
  ambiguous matches are narrowed by parent parameters or rejected
- Add campaign_territory_id lookup via observation.campaign_location
- Auto name sampling_log and observation_log (name and tag)
- Reject name/alias/tag containing "_" or "@" unless it equals the
  auto_name result; manage_geolocation name is exempt
- Update LUCAS prepare scripts and Excel sources to use auto naming

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/lucas/import_data/dataset_meta/excel/campaign.xlsx
+++ b/lucas/import_data/dataset_meta/excel/campaign.xlsx
@@ -20,12 +20,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="46">
   <si>
     <t xml:space="preserve">dataset_id__dataset_name</t>
   </si>
   <si>
-    <t xml:space="preserve">name</t>
+    <t xml:space="preserve">datetime_tag</t>
   </si>
   <si>
     <t xml:space="preserve">display_name</t>
@@ -103,9 +103,6 @@
     <t xml:space="preserve">lucas</t>
   </si>
   <si>
-    <t xml:space="preserve">lucas_eu_2009</t>
-  </si>
-  <si>
     <t xml:space="preserve">LUCAS 2009</t>
   </si>
   <si>
@@ -133,10 +130,7 @@
     <t xml:space="preserve">m</t>
   </si>
   <si>
-    <t xml:space="preserve">foss xds rca,lucas-wetlab-2009</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lucas_eu_2015</t>
+    <t xml:space="preserve">foss xds rca,lucas wetlab 2009</t>
   </si>
   <si>
     <t xml:space="preserve">LUCAS 2015</t>
@@ -145,7 +139,7 @@
     <t xml:space="preserve">https://esdac.jrc.ec.europa.eu/content/lucas2015-topsoil-data</t>
   </si>
   <si>
-    <t xml:space="preserve">foss xds rca,lucas-wetlab-2015</t>
+    <t xml:space="preserve">foss xds rca,lucas wetlab 2015</t>
   </si>
   <si>
     <t xml:space="preserve">biogeo16</t>
@@ -252,7 +246,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -265,19 +259,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -468,7 +454,7 @@
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="33.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="27.64"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="23.63"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="1" width="24.04"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="23.83"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="24.04"/>
@@ -477,7 +463,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="15.32"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="20.93"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="20.93"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="25.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="1" width="14.62"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="1" width="53.28"/>
   </cols>
@@ -566,17 +552,17 @@
       <c r="A2" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="1" t="n">
+        <v>2009</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>29</v>
-      </c>
       <c r="E2" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>20090501</v>
@@ -585,51 +571,51 @@
         <v>20091031</v>
       </c>
       <c r="H2" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="J2" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>31</v>
       </c>
       <c r="N2" s="1" t="n">
         <v>1</v>
       </c>
       <c r="T2" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="U2" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="U2" s="1" t="s">
+      <c r="V2" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="V2" s="1" t="s">
+      <c r="W2" s="1" t="s">
         <v>34</v>
-      </c>
-      <c r="W2" s="1" t="s">
-        <v>35</v>
       </c>
       <c r="X2" s="1" t="n">
         <v>1000</v>
       </c>
       <c r="Y2" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="Z2" s="1" t="s">
         <v>36</v>
-      </c>
-      <c r="Z2" s="1" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>38</v>
+      <c r="B3" s="1" t="n">
+        <v>2015</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F3" s="1" t="n">
         <v>20150501</v>
@@ -637,52 +623,52 @@
       <c r="G3" s="1" t="n">
         <v>20151031</v>
       </c>
-      <c r="H3" s="4" t="s">
-        <v>40</v>
+      <c r="H3" s="3" t="s">
+        <v>38</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N3" s="1" t="n">
         <v>1</v>
       </c>
       <c r="T3" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="U3" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="U3" s="1" t="s">
+      <c r="V3" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="V3" s="1" t="s">
+      <c r="W3" s="1" t="s">
         <v>34</v>
-      </c>
-      <c r="W3" s="1" t="s">
-        <v>35</v>
       </c>
       <c r="X3" s="1" t="n">
         <v>1000</v>
       </c>
       <c r="Y3" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="Z3" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>42</v>
+        <v>40</v>
+      </c>
+      <c r="B4" s="1" t="n">
+        <v>2016</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F4" s="1" t="n">
         <v>20160331</v>
@@ -691,34 +677,34 @@
         <v>20261231</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="J4" s="6" t="s">
-        <v>45</v>
+        <v>42</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>43</v>
       </c>
       <c r="S4" s="1" t="n">
         <v>1</v>
       </c>
       <c r="T4" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="U4" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="U4" s="1" t="s">
+      <c r="V4" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="V4" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="W4" s="0" t="s">
-        <v>46</v>
+      <c r="W4" s="1" t="s">
+        <v>44</v>
       </c>
       <c r="X4" s="1" t="n">
         <v>1000</v>
       </c>
       <c r="Y4" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="Z4" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Anchor campaign in place and sampling_log in time
Campaign is now named from dataset + territory (+ optional site), and
sampling_log from campaign + datetime_tag. LUCAS 2009 and 2015 become one
campaign (lucas_eu) with two sampling_logs (lucas_eu_2009, lucas_eu_2015).

- auto_name: optional concat arguments (site?) are dropped with their
  separator when empty; territory and datetime_tag get strict null values
  ('0' in tags, 'no location' / 'no date' in names)
- auto_name: values in a tag may only hold a-z, 0-9, '.' and '-';
  datetime_tag must be 0 or YYYY, YYYYMM, YYYYMMDD or YYYYMMDDhhmmss
- find_record also searches single-column UNIQUE text columns (e.g.
  territory iso code 'eu') and logs failed searches instead of crashing
- removed the campaign_territory_id special case
- campaign table drops datetime_tag; sampling_log gains datetime_tag,
  display_name and url
- prepare scripts and campaign.xlsx follow the new names

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/lucas/import_data/dataset_meta/excel/campaign.xlsx
+++ b/lucas/import_data/dataset_meta/excel/campaign.xlsx
@@ -20,14 +20,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="43">
   <si>
     <t xml:space="preserve">dataset_id__dataset_name</t>
   </si>
   <si>
-    <t xml:space="preserve">datetime_tag</t>
-  </si>
-  <si>
     <t xml:space="preserve">display_name</t>
   </si>
   <si>
@@ -103,7 +100,7 @@
     <t xml:space="preserve">lucas</t>
   </si>
   <si>
-    <t xml:space="preserve">LUCAS 2009</t>
+    <t xml:space="preserve">LUCAS EU</t>
   </si>
   <si>
     <t xml:space="preserve">inherit</t>
@@ -118,9 +115,6 @@
     <t xml:space="preserve">EU</t>
   </si>
   <si>
-    <t xml:space="preserve">Europe</t>
-  </si>
-  <si>
     <t xml:space="preserve">geographic</t>
   </si>
   <si>
@@ -133,9 +127,6 @@
     <t xml:space="preserve">foss xds rca,lucas wetlab 2009</t>
   </si>
   <si>
-    <t xml:space="preserve">LUCAS 2015</t>
-  </si>
-  <si>
     <t xml:space="preserve">https://esdac.jrc.ec.europa.eu/content/lucas2015-topsoil-data</t>
   </si>
   <si>
@@ -145,7 +136,7 @@
     <t xml:space="preserve">biogeo16</t>
   </si>
   <si>
-    <t xml:space="preserve">EU BIOGEO 2016</t>
+    <t xml:space="preserve">EU BIOGEO</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.eea.europa.eu/en/datahub/datahubitem-view/11db8d14-f167-4cd5-9205-95638dfd9618</t>
@@ -450,22 +441,21 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Z4"/>
+  <dimension ref="A1:Y4"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="33.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="23.63"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="1" width="24.04"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="23.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="24.04"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="23.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="23.63"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="15.32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="20.93"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="20.93"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="25.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="1" width="14.62"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="1" width="53.28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="24.04"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="23.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="24.04"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="23.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="23.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="15.32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="20.93"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="20.93"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="25.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="24" style="1" width="14.62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="1" width="53.28"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -541,175 +531,157 @@
       <c r="X1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" s="2" t="s">
         <v>24</v>
-      </c>
-      <c r="Z1" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>26</v>
-      </c>
-      <c r="B2" s="1" t="n">
-        <v>2009</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>27</v>
       </c>
       <c r="D2" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E2" s="1" t="n">
+        <v>20090501</v>
+      </c>
+      <c r="F2" s="1" t="n">
+        <v>20091031</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="E2" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="F2" s="1" t="n">
-        <v>20090501</v>
-      </c>
-      <c r="G2" s="1" t="n">
-        <v>20091031</v>
-      </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="M2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="S2" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="N2" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="T2" s="1" t="s">
+      <c r="T2" s="1"/>
+      <c r="U2" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="U2" s="1" t="s">
+      <c r="V2" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="V2" s="1" t="s">
+      <c r="W2" s="1" t="n">
+        <v>1000</v>
+      </c>
+      <c r="X2" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="W2" s="1" t="s">
+      <c r="Y2" s="1" t="s">
         <v>34</v>
-      </c>
-      <c r="X2" s="1" t="n">
-        <v>1000</v>
-      </c>
-      <c r="Y2" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="Z2" s="1" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B3" s="1" t="n">
-        <v>2015</v>
-      </c>
       <c r="C3" s="1" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
+      </c>
+      <c r="E3" s="1" t="n">
+        <v>20150501</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>20150501</v>
-      </c>
-      <c r="G3" s="1" t="n">
         <v>20151031</v>
       </c>
-      <c r="H3" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="J3" s="1" t="s">
+      <c r="G3" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="M3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="S3" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="N3" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="T3" s="1" t="s">
+      <c r="T3" s="1"/>
+      <c r="U3" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="U3" s="1" t="s">
+      <c r="V3" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="V3" s="1" t="s">
+      <c r="W3" s="1" t="n">
+        <v>1000</v>
+      </c>
+      <c r="X3" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="W3" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="X3" s="1" t="n">
-        <v>1000</v>
-      </c>
       <c r="Y3" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="Z3" s="1" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E4" s="1" t="n">
+        <v>20160331</v>
+      </c>
+      <c r="F4" s="1" t="n">
+        <v>20261231</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I4" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="B4" s="1" t="n">
-        <v>2016</v>
-      </c>
-      <c r="C4" s="1" t="s">
+      <c r="R4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="S4" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="T4" s="1"/>
+      <c r="U4" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="V4" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D4" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="F4" s="1" t="n">
-        <v>20160331</v>
-      </c>
-      <c r="G4" s="1" t="n">
-        <v>20261231</v>
-      </c>
-      <c r="H4" s="1" t="s">
+      <c r="W4" s="1" t="n">
+        <v>1000</v>
+      </c>
+      <c r="X4" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y4" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="J4" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="S4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="T4" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="U4" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="V4" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="W4" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="X4" s="1" t="n">
-        <v>1000</v>
-      </c>
-      <c r="Y4" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="Z4" s="1" t="s">
-        <v>45</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="H3" r:id="rId1" display="https://esdac.jrc.ec.europa.eu/content/lucas2015-topsoil-data"/>
+    <hyperlink ref="G3" r:id="rId1" display="https://esdac.jrc.ec.europa.eu/content/lucas2015-topsoil-data"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.025" bottom="1.025" header="0.7875" footer="0.7875"/>

</xml_diff>